<commit_message>
Lab 01. Review Form: Architect. Design Phase Defects
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cosmi\OneDrive\Desktop\FMI-UBB\Anul_III\Semestrul_II\VVSS\Laborator\LabVVSS\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDF422FD-C07C-43D3-B30D-68CD5525CDE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5E4F53-61E2-479A-B453-CCDE8D3EA9A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="650" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -210,19 +210,56 @@
   </si>
   <si>
     <t>Popovici Cosmina-Maria, Petri Dan, Preduca Matei</t>
+  </si>
+  <si>
+    <t>05.03.2026</t>
+  </si>
+  <si>
+    <t>A01</t>
+  </si>
+  <si>
+    <t>A02</t>
+  </si>
+  <si>
+    <t>A05</t>
+  </si>
+  <si>
+    <t>A06</t>
+  </si>
+  <si>
+    <t>Clasele de Validare și de Excepții sunt definite, dar nu sunt integrate în arhitectura aplicației (nu sunt folosite).</t>
+  </si>
+  <si>
+    <t>Se folosesc șabloanele: Repository, MVC.</t>
+  </si>
+  <si>
+    <t>Ar fi de preferat ca pentru fiecare tip de Repository să existe o interfață specifică, care să o extindă pe cea generală. În timp se poate încălca principiul Segregării Iterfețelor din SOLID.</t>
+  </si>
+  <si>
+    <t>Partiționarea/ arhitectura pachetelor este inconsitentă. Se amestecă separarea pe nivele/ layere (model, business, persistence, ui) cu cea pe funcționalități (există pachete separate pentru: export, receipt, reports). Conform cerinței, arhitectura trebuie să fie una stratificată clar, astfel, clasa DailyReportService din modulul reports, ar trebui pusă în cel de Serivce, iar modulul reports nu ar trebui să existe.</t>
+  </si>
+  <si>
+    <t>30min</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -408,91 +445,92 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -549,6 +587,55 @@
         <a:xfrm>
           <a:off x="6987540" y="1478281"/>
           <a:ext cx="5721735" cy="3498688"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>579592</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>292519</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>118969</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F59392C-7A22-01BB-1197-2A7637B74461}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7094692" y="1165860"/>
+          <a:ext cx="5496507" cy="4477609"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -868,19 +955,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -904,10 +991,10 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="26"/>
+      <c r="E4" s="31"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -922,10 +1009,10 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="28"/>
+      <c r="E5" s="33"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -941,19 +1028,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="E6" s="23"/>
+      <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="23"/>
+      <c r="E7" s="28"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -970,102 +1057,102 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="B10" s="37">
+      <c r="B10" s="23">
         <v>1</v>
       </c>
-      <c r="C10" s="38" t="s">
+      <c r="C10" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="38" t="s">
+      <c r="D10" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="25" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="72" x14ac:dyDescent="0.3">
-      <c r="B11" s="37">
+      <c r="B11" s="23">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="38" t="s">
+      <c r="C11" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="39" t="s">
+      <c r="E11" s="25" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B12" s="37">
+      <c r="B12" s="23">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="38" t="s">
+      <c r="C12" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="38" t="s">
+      <c r="D12" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="E12" s="39" t="s">
+      <c r="E12" s="25" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B13" s="37">
+      <c r="B13" s="23">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="38" t="s">
+      <c r="C13" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="38" t="s">
+      <c r="D13" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="39" t="s">
+      <c r="E13" s="25" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B14" s="37">
+      <c r="B14" s="23">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="38" t="s">
+      <c r="C14" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="E14" s="39" t="s">
+      <c r="E14" s="25" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="37">
+      <c r="B15" s="23">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="38" t="s">
+      <c r="C15" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="38"/>
-      <c r="E15" s="39" t="s">
+      <c r="D15" s="24"/>
+      <c r="E15" s="25" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B16" s="37">
+      <c r="B16" s="23">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="38" t="s">
+      <c r="C16" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="38"/>
-      <c r="E16" s="39" t="s">
+      <c r="D16" s="24"/>
+      <c r="E16" s="25" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1196,19 +1283,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1221,51 +1308,67 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
+      <c r="I3" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="26" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="34"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="I4" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="26" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="31"/>
+      <c r="E5" s="36"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
+      <c r="I5" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" s="26" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
+      <c r="D6" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
+      <c r="D7" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="28"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1281,40 +1384,56 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E10" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>61</v>
+      </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E11" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="131.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
+      <c r="E12" s="27" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
@@ -1438,7 +1557,9 @@
         <v>8</v>
       </c>
       <c r="D28" s="12"/>
-      <c r="E28" s="1"/>
+      <c r="E28" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1451,6 +1572,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1477,19 +1599,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1509,10 +1631,10 @@
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="37"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1523,10 +1645,10 @@
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="34"/>
+      <c r="E5" s="39"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1538,15 +1660,15 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1795,19 +1917,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1827,8 +1949,8 @@
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1839,8 +1961,8 @@
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1852,8 +1974,8 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
       <c r="F6" s="20"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -2083,11 +2205,11 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="35" t="s">
+      <c r="C32" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="41"/>
       <c r="F32" s="18"/>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Lab 01. Version 01.
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cosmi\OneDrive\Desktop\FMI-UBB\Anul_III\Semestrul_II\VVSS\Laborator\LabVVSS\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5E4F53-61E2-479A-B453-CCDE8D3EA9A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E316130C-4E09-403D-9EBB-E3CFB55BE089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="650" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="108">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -240,19 +240,312 @@
   </si>
   <si>
     <t>30min</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>Nu există legătură între Product și Rețeta lui. Avem listă de Prudse și Rețete dar nu știm cum sunt asociate, „care și cum vin”.</t>
+  </si>
+  <si>
+    <t>C06</t>
+  </si>
+  <si>
+    <t>La update ar trebui să se modifice doar ce există. Dacă entity, nu există deja, ar trebui aruncată o eroare, în care să se anunțe utilizatorul că nu există entitate pe care vrea să o modifice.</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>Prețul ar putea fi zero, dacă e ceva din partea casei. (ProductValidator).</t>
+  </si>
+  <si>
+    <t>StocService (line:73)</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>Nu se fac validări.</t>
+  </si>
+  <si>
+    <t>DrinkShopController (line: 233)</t>
+  </si>
+  <si>
+    <t>1h</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Se aruncă partea zecimală
+Dacă ai stoc 10.5 și consumi 0.7, rezultatul devine 9.8, dar tu îl convertești la int → 9.
+Asta duce la pierdere de precizie și stoc incorect.
+Stoc.getCantitate() este double, dar este tratat ca int
+Dacă ingredientele pot avea cantități fracționale (de ex. 0.5 litri, 0.2 kg), conversia la int este greșită.*</t>
+  </si>
+  <si>
+    <t>Ultimul parametrul al constructorului ar trebui să se numească stocRepo, pentru a fi sugestiv.*</t>
+  </si>
+  <si>
+    <t>ID-ul rețetei este generat ca size + 1.
+Dacă ștergi o rețetă, se generează un ID duplicat.*</t>
+  </si>
+  <si>
+    <t>Popovici Cosmina-Maria,Petri Dan,Preduca Matei</t>
+  </si>
+  <si>
+    <t>SonarQube</t>
+  </si>
+  <si>
+    <t>OrderItem, line 7</t>
+  </si>
+  <si>
+    <t>Make non-static "product" transient or serializable.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">public class </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Product</t>
+    </r>
+  </si>
+  <si>
+    <t>Add at least one assertion in this case</t>
+  </si>
+  <si>
+    <t>ProductTest</t>
+  </si>
+  <si>
+    <t>package drinkshop.domain;
+import org.junit.jupiter.api.AfterEach;
+import org.junit.jupiter.api.BeforeEach;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.*;
+class ProductTest {
+    Product product;
+    @BeforeEach
+    void setUp() {
+        product =new Product(100, "Limonada", 10.0, CategorieBautura.JUICE, TipBautura.WATER_BASED);
+    }
+    @AfterEach
+    void tearDown() {
+        product = null;
+    }
+    @Test
+    void getId() {
+        assertEquals(100, product.getId());
+    }
+    @Test
+    void getNume() {
+        assertEquals("Limonada", product.getNume());
+    }
+    @Test
+    void getPret() {
+        assertEquals(10.0, product.getPret());
+    }
+    @Test
+    void getCategorie() {
+        assertEquals(CategorieBautura.JUICE, product.getCategorie());
+    }
+    @Test
+    void setCategorie() {
+        product.setCategorie(CategorieBautura.SMOOTHIE);
+        assertEquals(CategorieBautura.SMOOTHIE, product.getCategorie());
+    }
+    @Test
+    void getTip() {
+        assertEquals(TipBautura.WATER_BASED, product.getTip());
+    }
+    @Test
+    void setTip() {
+        product.setTip(TipBautura.BASIC);
+        assertEquals(TipBautura.BASIC, product.getTip());
+    }
+    @Test
+    void setNume() {
+        product.setNume("newLimonada");
+        assertEquals("newLimonada", product.getNume());
+    }
+    @Test
+    void setPret() {
+        product.setPret(10.05);
+        assertEquals(10.05, product.getPret());
+    }
+    @Test
+    void testToString() {
+        assertEquals("Limonada (JUICE, WATER_BASED) - 10.0 lei", product.toString());
+    }
+}</t>
+  </si>
+  <si>
+    <t>public class Product implements Serializable</t>
+  </si>
+  <si>
+    <t>package drinkshop.domain;
+import org.junit.jupiter.api.AfterEach;
+import org.junit.jupiter.api.BeforeEach;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.*;
+class ProductTest {
+    Product product;
+    @BeforeEach
+    void setUp() {
+        product =new Product(100, "Limonada", 10.0, CategorieBautura.JUICE, TipBautura.WATER_BASED);
+    }
+    @AfterEach
+    void tearDown() {
+        product = null;
+    }
+    @Test
+    void getId() {
+        assert 100 == product.getId();
+    }
+    @Test
+    void getNume() {
+        assert "Limonada".equals(product.getNume());
+    }
+    @Test
+    void getPret() {
+        assert 10.0 == product.getPret();
+    }
+    @Test
+    void getCategorie() {
+        assert CategorieBautura.JUICE.equals(product.getCategorie());
+    }
+    @Test
+    void setCategorie() {
+        product.setCategorie(CategorieBautura.SMOOTHIE);
+        assert CategorieBautura.SMOOTHIE.equals(product.getCategorie());
+    }
+    @Test
+    void getTip() {
+        assert TipBautura.WATER_BASED.equals(product.getTip());
+    }
+    @Test
+    void setTip() {
+        product.setTip(TipBautura.BASIC);
+        assert TipBautura.BASIC.equals(product.getTip());
+    }
+    @Test
+    void setNume() {
+        product.setNume("newLimonada");
+        assert "newLimonada".equals(product.getNume());
+    }
+    @Test
+    void setPret() {
+        product.setPret(10.05);
+        assert 10.05 == product.getPret();
+    }
+    @Test
+    void testToString() {
+        System.out.println(product.toString());
+        assert "Limonada (JUICE, WATER_BASED) - 10.0 lei".equals(product.toString());
+    }
+}</t>
+  </si>
+  <si>
+    <t>Update this method so that its implementation is not identical to "save" on line 26.</t>
+  </si>
+  <si>
+    <t>AbstractRepository, 37-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+    public E update(E entity) {
+        entities.put(getId(entity), entity);
+        return entity;
+    }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+public E update(E entity) {
+    ID id = getId(entity);
+    // dacă nu există, nu facem update
+    if (!entities.containsKey(id)) {
+        return null; // sau poți arunca o excepție
+    }
+    // înlocuim doar dacă exista
+    entities.put(id, entity);
+    return entity;
+}</t>
+  </si>
+  <si>
+    <t>CsvExporter, 14</t>
+  </si>
+  <si>
+    <t>Add a private constructor to hide the implicit public one.</t>
+  </si>
+  <si>
+    <t>nu era</t>
+  </si>
+  <si>
+    <t>private CsvExporter(){
+    }</t>
+  </si>
+  <si>
+    <t>Use "isEmpty()" to check whether a "StringBuilder" is empty or not.</t>
+  </si>
+  <si>
+    <t>FileOrderRepository, 59</t>
+  </si>
+  <si>
+    <t>if (sb.length() &gt; 0) {
+                sb.append("|");
+            }</t>
+  </si>
+  <si>
+    <t>if (sb.isEmpty()) {
+                sb.append("|");
+            }</t>
+  </si>
+  <si>
+    <t>A "NullPointerException" could be thrown; "ingrediente" is nullable here.</t>
+  </si>
+  <si>
+    <t>RetetaValidator, 23</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> if (ingrediente == null || ingrediente.isEmpty())
+            errors.accumulateAndGet("Ingrediente empty!\n", String::concat);
+        ingrediente.stream()
+                .filter(entry -&gt; entry.getCantitate() &lt;= 0)
+                .forEach(entry -&gt; {
+                    errors.accumulateAndGet("[" + entry.getDenumire() + "]"+ "cantitate negativa sau zero", String::concat);
+                });</t>
+  </si>
+  <si>
+    <t>if (ingrediente != null) {
+            ingrediente.stream()
+                    .filter(entry -&gt; entry.getCantitate() &lt;= 0)
+                    .forEach(entry -&gt; {
+                        errors.accumulateAndGet("[" + entry.getDenumire() + "]" + "cantitate negativa sau zero", String::concat);
+                    });
+        }</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -344,6 +637,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFBCBEC4"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFCF8E6D"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="5">
@@ -445,92 +750,108 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -610,7 +931,7 @@
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>292519</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>118969</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -636,6 +957,275 @@
         <a:xfrm>
           <a:off x="7094692" y="1165860"/>
           <a:ext cx="5496507" cy="4477609"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>117186</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>350520</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>316499</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEC49B75-690D-A171-DA8F-C9A475B87D43}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7363806" y="1493520"/>
+          <a:ext cx="5117754" cy="4797059"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2461713</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>876300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5036D883-A9FC-E30C-26BB-D85DEB6571B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2560321" y="1661160"/>
+          <a:ext cx="2461712" cy="876300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2484121</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>467923</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1C672197-B0F2-5EB1-EF57-4C777DD10E2E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2560321" y="3314700"/>
+          <a:ext cx="2484120" cy="467923"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2501574</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3062CF3-6305-65F1-23B5-53E591478CD4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2567940" y="3863340"/>
+          <a:ext cx="2493954" cy="144780"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2446021</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>785201</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5DE7CA2F-F878-FC68-80A6-D0DAE4B768E4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2560321" y="5669280"/>
+          <a:ext cx="2446020" cy="785201"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2446020</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>257211</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E5F62A5-86F5-1F1F-C3DD-1C74DD1819C7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2560320" y="6705600"/>
+          <a:ext cx="2446020" cy="257211"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -938,7 +1528,7 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="6"/>
     <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
@@ -950,24 +1540,24 @@
     <col min="11" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.6">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="29" t="s">
+      <c r="H1" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -976,7 +1566,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
@@ -987,14 +1577,14 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10">
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="31"/>
+      <c r="E4" s="35"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1005,14 +1595,14 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="33"/>
+      <c r="E5" s="37"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1023,26 +1613,26 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="E6" s="28"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E6" s="32"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="28"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E7" s="32"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1056,7 +1646,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="172.8">
       <c r="B10" s="23">
         <v>1</v>
       </c>
@@ -1070,7 +1660,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="72">
       <c r="B11" s="23">
         <f>B10+1</f>
         <v>2</v>
@@ -1085,7 +1675,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10">
       <c r="B12" s="23">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
@@ -1100,7 +1690,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="28.8">
       <c r="B13" s="23">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1115,7 +1705,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="57.6">
       <c r="B14" s="23">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1130,7 +1720,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="57.6">
       <c r="B15" s="23">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1143,7 +1733,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="43.2">
       <c r="B16" s="23">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1156,7 +1746,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1165,7 +1755,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1174,7 +1764,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1183,7 +1773,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1192,7 +1782,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1201,7 +1791,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1210,7 +1800,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1219,7 +1809,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1228,7 +1818,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1237,7 +1827,7 @@
       <c r="D25" s="3"/>
       <c r="E25" s="15"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5">
       <c r="C27" s="11" t="s">
         <v>8</v>
       </c>
@@ -1267,7 +1857,7 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="6"/>
     <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
@@ -1278,24 +1868,24 @@
     <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.6">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="29" t="s">
+      <c r="H1" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1304,7 +1894,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
@@ -1315,14 +1905,14 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="34"/>
+      <c r="E4" s="38"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1333,14 +1923,14 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="36"/>
+      <c r="E5" s="40"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1351,26 +1941,26 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="E6" s="28"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E6" s="32"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="E7" s="28"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E7" s="32"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1384,7 +1974,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="57.6">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1396,7 +1986,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="43.2">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1409,7 +1999,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="131.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="131.4" customHeight="1">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
@@ -1422,7 +2012,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1435,16 +2025,20 @@
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="43.2">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>68</v>
+      </c>
       <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E14" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1453,7 +2047,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1462,7 +2056,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1471,7 +2065,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1480,7 +2074,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1489,7 +2083,7 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1498,7 +2092,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1507,7 +2101,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1516,7 +2110,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1525,7 +2119,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1534,7 +2128,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1543,7 +2137,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1552,7 +2146,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5">
       <c r="C28" s="11" t="s">
         <v>8</v>
       </c>
@@ -1581,37 +2175,37 @@
   <sheetPr>
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J31"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="6"/>
     <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
     <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="18" style="6" customWidth="1"/>
+    <col min="4" max="4" width="36.6640625" style="6" customWidth="1"/>
     <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
     <col min="6" max="8" width="8.88671875" style="6"/>
     <col min="9" max="9" width="26.77734375" style="6" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.6">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="29" t="s">
+      <c r="H1" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1620,57 +2214,73 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I3" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="37"/>
+      <c r="E4" s="41"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I4" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="39"/>
+      <c r="E5" s="43"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I5" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D6" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="E6" s="32"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D7" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="32"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1684,60 +2294,86 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="72.599999999999994" customHeight="1">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="41.4" customHeight="1">
       <c r="B11" s="3">
-        <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E11" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="144">
       <c r="B12" s="3">
-        <f t="shared" ref="B12:B30" si="0">B11+1</f>
+        <f t="shared" ref="B12:B29" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="67.2" customHeight="1">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E13" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>70</v>
+      </c>
       <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E14" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="31.8" customHeight="1">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="29" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1746,7 +2382,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1755,43 +2391,43 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
+      <c r="D18" s="1"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
+      <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C20" s="1"/>
-      <c r="D20" s="2"/>
+      <c r="D20" s="1"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
+      <c r="D21" s="2"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1800,7 +2436,7 @@
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1809,7 +2445,7 @@
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1818,34 +2454,34 @@
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C25" s="1"/>
-      <c r="D25" s="2"/>
+      <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="D26" s="2"/>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="2:5">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="2:5">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1854,7 +2490,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1863,21 +2499,14 @@
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B30" s="3">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="C30" s="1"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C32" s="11" t="s">
+    <row r="31" spans="2:5">
+      <c r="C31" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D32" s="12"/>
-      <c r="E32" s="1"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="1" t="s">
+        <v>78</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1890,6 +2519,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1899,37 +2529,37 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="6"/>
     <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.88671875" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="22.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="70.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="62.44140625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="51" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="8.88671875" style="6"/>
     <col min="9" max="9" width="26.77734375" style="6" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.6">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="29" t="s">
+      <c r="H1" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1938,47 +2568,65 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I3" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
+      <c r="D4" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="41"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I4" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
+      <c r="D5" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="32"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I5" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
+      <c r="D6" s="46" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="47"/>
       <c r="F6" s="20"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1995,66 +2643,114 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="39" customHeight="1">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E10" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="F10" s="30" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="409.2" customHeight="1">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="187.2">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>92</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="43.2">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>97</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="43.2">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>100</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="129.6">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2064,7 +2760,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2074,7 +2770,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2084,7 +2780,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2094,7 +2790,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2104,7 +2800,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2114,7 +2810,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2124,7 +2820,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2134,7 +2830,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2144,7 +2840,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2154,7 +2850,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2164,7 +2860,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2174,7 +2870,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2184,7 +2880,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2194,7 +2890,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -2204,15 +2900,15 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="40" t="s">
+    <row r="32" spans="2:6">
+      <c r="C32" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="41"/>
-      <c r="E32" s="41"/>
+      <c r="D32" s="45"/>
+      <c r="E32" s="45"/>
       <c r="F32" s="18"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="6:6">
       <c r="F35" s="21"/>
     </row>
   </sheetData>

</xml_diff>